<commit_message>
Added trianing steps excel
</commit_message>
<xml_diff>
--- a/steps.xlsx
+++ b/steps.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://toagi-my.sharepoint.com/personal/srinivas_devi_core42_ai/Documents/Desktop/Backup/Github/Sample3/git-team-playground/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_F25DC773A252ABDACC104896B11B47585ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF7D654-44C0-49D9-9DB8-01B810DA3ADD}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_F25DC773A252ABDACC104896B11B47585ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{600A0BAA-4738-4BAD-B0D1-95E6D9CAC7C8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>git fetch</t>
   </si>
@@ -34,6 +34,15 @@
   </si>
   <si>
     <t>git switch -c features/update-developer1</t>
+  </si>
+  <si>
+    <t>git push -u origin feature/update-developer1</t>
+  </si>
+  <si>
+    <t>git add steps.xslx</t>
+  </si>
+  <si>
+    <t>git commit -m "Added trianing steps.xlsx"</t>
   </si>
 </sst>
 </file>
@@ -351,10 +360,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -370,6 +379,21 @@
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>